<commit_message>
Human readable version of feature set saved to excel file with date of each event formatted as a string
</commit_message>
<xml_diff>
--- a/mfc_features.xlsx
+++ b/mfc_features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uob-my.sharepoint.com/personal/hp12384_bristol_ac_uk/Documents/Projects/APEX/APEX_WP2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_2299CC05A0D764E4975C3285521D731F78C745D2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E2DEC22-EE13-C54C-80F9-92A0711F95E1}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_36C5A469B1942586A8DAF0BA92C89005C29E96B8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0620DFDC-26A5-E646-B488-99B69FC79DA3}"/>
   <bookViews>
-    <workbookView xWindow="-29500" yWindow="-860" windowWidth="28500" windowHeight="19700" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COD date time index" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="42">
   <si>
     <t>Date</t>
   </si>
@@ -66,6 +66,93 @@
   </si>
   <si>
     <t>12) 20*30 -3</t>
+  </si>
+  <si>
+    <t>24/07/2024</t>
+  </si>
+  <si>
+    <t>29/07/2024</t>
+  </si>
+  <si>
+    <t>02/08/2024</t>
+  </si>
+  <si>
+    <t>06/08/2024</t>
+  </si>
+  <si>
+    <t>08/08/2024</t>
+  </si>
+  <si>
+    <t>16/09/2024</t>
+  </si>
+  <si>
+    <t>24/09/2024</t>
+  </si>
+  <si>
+    <t>02/10/2024</t>
+  </si>
+  <si>
+    <t>10/10/2024</t>
+  </si>
+  <si>
+    <t>12/10/2024</t>
+  </si>
+  <si>
+    <t>16/10/2024</t>
+  </si>
+  <si>
+    <t>25/10/2024</t>
+  </si>
+  <si>
+    <t>10/12/2024</t>
+  </si>
+  <si>
+    <t>07/02/2025</t>
+  </si>
+  <si>
+    <t>11/02/2025</t>
+  </si>
+  <si>
+    <t>14/02/2025</t>
+  </si>
+  <si>
+    <t>21/02/2025</t>
+  </si>
+  <si>
+    <t>24/02/2025</t>
+  </si>
+  <si>
+    <t>02/04/2025</t>
+  </si>
+  <si>
+    <t>03/04/2025</t>
+  </si>
+  <si>
+    <t>04/04/2025</t>
+  </si>
+  <si>
+    <t>28/04/2025</t>
+  </si>
+  <si>
+    <t>30/04/2025</t>
+  </si>
+  <si>
+    <t>07/05/2025</t>
+  </si>
+  <si>
+    <t>08/05/2025</t>
+  </si>
+  <si>
+    <t>09/05/2025</t>
+  </si>
+  <si>
+    <t>12/05/2025</t>
+  </si>
+  <si>
+    <t>13/05/2025</t>
+  </si>
+  <si>
+    <t>18/05/2025</t>
   </si>
 </sst>
 </file>
@@ -411,6 +498,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -454,8 +544,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>45497.456319444442</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2" s="1">
         <v>45497.444166666668</v>
@@ -495,8 +585,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>45502.568819444437</v>
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3" s="1">
         <v>45502.557013888887</v>
@@ -536,8 +626,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>45506.432141203702</v>
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4" s="1">
         <v>45506.421377314808</v>
@@ -577,8 +667,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>45510.431689814817</v>
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5" s="1">
         <v>45510.420578703714</v>
@@ -618,8 +708,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>45512.469583333332</v>
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6" s="1">
         <v>45512.460555555554</v>
@@ -659,8 +749,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>45551.438842592594</v>
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7" s="1">
         <v>45551.427384259259</v>
@@ -700,8 +790,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>45559.396516203713</v>
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8" s="1">
         <v>45559.396516203713</v>
@@ -741,8 +831,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>45567.486678240741</v>
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9" s="1">
         <v>45567.475219907406</v>
@@ -782,8 +872,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>45575.428530092591</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10" s="1">
         <v>45575.417071759257</v>
@@ -823,8 +913,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>45577.514988425923</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11" s="1">
         <v>45577.504918981482</v>
@@ -864,8 +954,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>45581.431863425933</v>
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12" s="1">
         <v>45581.4221412037</v>
@@ -905,8 +995,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>45590.521087962959</v>
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13" s="1">
         <v>45590.509282407409</v>
@@ -946,8 +1036,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>45636.426770833343</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14" s="1">
         <v>45636.417743055557</v>
@@ -987,8 +1077,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>45695.437777777777</v>
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15" s="1">
         <v>45695.426319444443</v>
@@ -1028,8 +1118,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>45699.435034722221</v>
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16" s="1">
         <v>45699.422881944447</v>
@@ -1069,8 +1159,8 @@
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>45702.570150462961</v>
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17" s="1">
         <v>45702.557650462957</v>
@@ -1110,8 +1200,8 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>45709.443043981482</v>
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18" s="1">
         <v>45709.429502314822</v>
@@ -1151,8 +1241,8 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>45712.429942129631</v>
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19" s="1">
         <v>45712.416400462957</v>
@@ -1192,8 +1282,8 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>45749.684745370367</v>
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20" s="1">
         <v>45749.671550925923</v>
@@ -1233,8 +1323,8 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>45750.456342592603</v>
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21" s="1">
         <v>45750.442800925928</v>
@@ -1274,8 +1364,8 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>45751.463090277779</v>
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22" s="1">
         <v>45751.450590277767</v>
@@ -1315,8 +1405,8 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>45775.660162037027</v>
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23" s="1">
         <v>45775.6487037037</v>
@@ -1356,8 +1446,8 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>45777.673206018517</v>
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24" s="1">
         <v>45777.661747685182</v>
@@ -1397,8 +1487,8 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>45784.682685185187</v>
+      <c r="A25" t="s">
+        <v>36</v>
       </c>
       <c r="B25" s="1">
         <v>45784.671226851853</v>
@@ -1438,8 +1528,8 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>45785.61341435185</v>
+      <c r="A26" t="s">
+        <v>37</v>
       </c>
       <c r="B26" s="1">
         <v>45785.601956018523</v>
@@ -1479,8 +1569,8 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>45786.607685185183</v>
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27" s="1">
         <v>45786.596226851849</v>
@@ -1520,8 +1610,8 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>45789.486319444448</v>
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28" s="1">
         <v>45789.474861111114</v>
@@ -1561,8 +1651,8 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>45790.532141203701</v>
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29" s="1">
         <v>45790.520335648151</v>
@@ -1602,8 +1692,8 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>45795.64603009259</v>
+      <c r="A30" t="s">
+        <v>41</v>
       </c>
       <c r="B30" s="1">
         <v>45795.63422453704</v>
@@ -1694,8 +1784,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>45497.456319444442</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
         <v>839</v>
@@ -1735,8 +1825,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>45502.568819444437</v>
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3">
         <v>180</v>
@@ -1776,8 +1866,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>45506.432141203702</v>
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4">
         <v>101</v>
@@ -1817,8 +1907,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>45510.431689814817</v>
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5">
         <v>47</v>
@@ -1858,8 +1948,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>45512.469583333332</v>
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6">
         <v>360</v>
@@ -1899,8 +1989,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>45551.438842592594</v>
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
         <v>900</v>
@@ -1940,8 +2030,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>45559.396516203713</v>
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8">
         <v>101</v>
@@ -1981,8 +2071,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>45567.486678240741</v>
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9">
         <v>360</v>
@@ -2022,8 +2112,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>45575.428530092591</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10">
         <v>185</v>
@@ -2063,8 +2153,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>45577.514988425923</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11">
         <v>79</v>
@@ -2104,8 +2194,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>45581.431863425933</v>
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12">
         <v>30</v>
@@ -2145,8 +2235,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>45590.521087962959</v>
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13">
         <v>270</v>
@@ -2186,8 +2276,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>45636.426770833343</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14">
         <v>900</v>
@@ -2227,8 +2317,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>45695.437777777777</v>
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15">
         <v>801</v>
@@ -2268,8 +2358,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>45699.435034722221</v>
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16">
         <v>785</v>
@@ -2309,8 +2399,8 @@
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>45702.570150462961</v>
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17">
         <v>312</v>
@@ -2350,8 +2440,8 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>45709.443043981482</v>
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18">
         <v>180</v>
@@ -2391,8 +2481,8 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>45712.429942129631</v>
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19">
         <v>76</v>
@@ -2432,8 +2522,8 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>45749.684745370367</v>
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20">
         <v>33</v>
@@ -2473,8 +2563,8 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>45750.456342592603</v>
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21">
         <v>162</v>
@@ -2514,8 +2604,8 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>45751.463090277779</v>
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22">
         <v>810</v>
@@ -2555,8 +2645,8 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>45775.660162037027</v>
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23">
         <v>844</v>
@@ -2596,8 +2686,8 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>45777.673206018517</v>
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24">
         <v>376</v>
@@ -2637,8 +2727,8 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>45784.682685185187</v>
+      <c r="A25" t="s">
+        <v>36</v>
       </c>
       <c r="B25">
         <v>198</v>
@@ -2678,8 +2768,8 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>45785.61341435185</v>
+      <c r="A26" t="s">
+        <v>37</v>
       </c>
       <c r="B26">
         <v>70</v>
@@ -2719,8 +2809,8 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>45786.607685185183</v>
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27">
         <v>817</v>
@@ -2760,8 +2850,8 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>45789.486319444448</v>
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28">
         <v>45</v>
@@ -2801,8 +2891,8 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>45790.532141203701</v>
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29">
         <v>182</v>
@@ -2842,8 +2932,8 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>45795.64603009259</v>
+      <c r="A30" t="s">
+        <v>41</v>
       </c>
       <c r="B30">
         <v>180</v>
@@ -2934,8 +3024,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>45497.456319444442</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2975,8 +3065,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>45502.568819444437</v>
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -3016,8 +3106,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>45506.432141203702</v>
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -3057,8 +3147,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>45510.431689814817</v>
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3098,8 +3188,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>45512.469583333332</v>
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -3139,8 +3229,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>45551.438842592594</v>
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
         <v>3</v>
@@ -3180,8 +3270,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>45559.396516203713</v>
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -3221,8 +3311,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>45567.486678240741</v>
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9">
         <v>3</v>
@@ -3262,8 +3352,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>45575.428530092591</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10">
         <v>3</v>
@@ -3303,8 +3393,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>45577.514988425923</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -3344,8 +3434,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>45581.431863425933</v>
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12">
         <v>3</v>
@@ -3385,8 +3475,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>45590.521087962959</v>
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13">
         <v>3</v>
@@ -3426,8 +3516,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>45636.426770833343</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14">
         <v>3</v>
@@ -3467,8 +3557,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>45695.437777777777</v>
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -3508,8 +3598,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>45699.435034722221</v>
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16">
         <v>3</v>
@@ -3549,8 +3639,8 @@
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>45702.570150462961</v>
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17">
         <v>3</v>
@@ -3590,8 +3680,8 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>45709.443043981482</v>
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18">
         <v>3</v>
@@ -3631,8 +3721,8 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>45712.429942129631</v>
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19">
         <v>3</v>
@@ -3672,8 +3762,8 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>45749.684745370367</v>
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20">
         <v>3</v>
@@ -3713,8 +3803,8 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>45750.456342592603</v>
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21">
         <v>3</v>
@@ -3754,8 +3844,8 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>45751.463090277779</v>
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -3795,8 +3885,8 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>45775.660162037027</v>
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23">
         <v>0.1</v>
@@ -3836,8 +3926,8 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>45777.673206018517</v>
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24">
         <v>0.1</v>
@@ -3877,8 +3967,8 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>45784.682685185187</v>
+      <c r="A25" t="s">
+        <v>36</v>
       </c>
       <c r="B25">
         <v>0.1</v>
@@ -3918,8 +4008,8 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>45785.61341435185</v>
+      <c r="A26" t="s">
+        <v>37</v>
       </c>
       <c r="B26">
         <v>0.1</v>
@@ -3959,8 +4049,8 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>45786.607685185183</v>
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27">
         <v>0.1</v>
@@ -4000,8 +4090,8 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>45789.486319444448</v>
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28">
         <v>0.1</v>
@@ -4041,8 +4131,8 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>45790.532141203701</v>
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29">
         <v>0.1</v>
@@ -4082,8 +4172,8 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>45795.64603009259</v>
+      <c r="A30" t="s">
+        <v>41</v>
       </c>
       <c r="B30">
         <v>0.1</v>
@@ -4174,8 +4264,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>45497.456319444442</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
         <v>162.982</v>
@@ -4215,8 +4305,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>45502.568819444437</v>
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3">
         <v>78.113</v>
@@ -4256,8 +4346,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>45506.432141203702</v>
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4">
         <v>42.896000000000001</v>
@@ -4297,8 +4387,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>45510.431689814817</v>
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5">
         <v>20.974</v>
@@ -4335,8 +4425,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>45512.469583333332</v>
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6">
         <v>100.102</v>
@@ -4376,8 +4466,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>45551.438842592594</v>
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
         <v>275.97899999999998</v>
@@ -4417,8 +4507,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>45559.396516203713</v>
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8">
         <v>9.1549999999999994</v>
@@ -4458,8 +4548,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>45567.486678240741</v>
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9">
         <v>84.486999999999995</v>
@@ -4499,8 +4589,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>45575.428530092591</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10">
         <v>3.7010000000000001</v>
@@ -4540,8 +4630,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>45577.514988425923</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11">
         <v>-5.4050000000000002</v>
@@ -4581,8 +4671,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>45581.431863425933</v>
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12">
         <v>-9.532</v>
@@ -4622,8 +4712,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>45590.521087962959</v>
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13">
         <v>41.942</v>
@@ -4663,8 +4753,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>45636.426770833343</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14">
         <v>87.986999999999995</v>
@@ -4704,8 +4794,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>45695.437777777777</v>
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15">
         <v>226.852</v>
@@ -4742,8 +4832,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>45699.435034722221</v>
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16">
         <v>330.64600000000002</v>
@@ -4783,8 +4873,8 @@
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>45702.570150462961</v>
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17">
         <v>224.16800000000001</v>
@@ -4824,8 +4914,8 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>45709.443043981482</v>
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18">
         <v>49.49</v>
@@ -4865,8 +4955,8 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>45712.429942129631</v>
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19">
         <v>27.222999999999999</v>
@@ -4906,8 +4996,8 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>45749.684745370367</v>
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20">
         <v>135.59100000000001</v>
@@ -4947,8 +5037,8 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>45750.456342592603</v>
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21">
         <v>158.90600000000001</v>
@@ -4988,8 +5078,8 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>45751.463090277779</v>
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22">
         <v>329.71300000000002</v>
@@ -5029,8 +5119,8 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>45775.660162037027</v>
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23">
         <v>68.546999999999997</v>
@@ -5070,8 +5160,8 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>45777.673206018517</v>
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24">
         <v>16.163</v>
@@ -5111,8 +5201,8 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>45784.682685185187</v>
+      <c r="A25" t="s">
+        <v>36</v>
       </c>
       <c r="B25">
         <v>13.675000000000001</v>
@@ -5152,8 +5242,8 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>45785.61341435185</v>
+      <c r="A26" t="s">
+        <v>37</v>
       </c>
       <c r="B26">
         <v>8.202</v>
@@ -5193,8 +5283,8 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>45786.607685185183</v>
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27">
         <v>23.042999999999999</v>
@@ -5234,8 +5324,8 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>45789.486319444448</v>
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28">
         <v>2.5590000000000002</v>
@@ -5275,8 +5365,8 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>45790.532141203701</v>
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29">
         <v>4.5090000000000003</v>
@@ -5316,8 +5406,8 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>45795.64603009259</v>
+      <c r="A30" t="s">
+        <v>41</v>
       </c>
       <c r="B30">
         <v>-0.42899999999999999</v>
@@ -5408,8 +5498,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>45497.456319444442</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
         <v>2.6563132324E-5</v>
@@ -5449,8 +5539,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>45502.568819444437</v>
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3">
         <v>6.1016407690000001E-6</v>
@@ -5490,8 +5580,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>45506.432141203702</v>
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4">
         <v>1.8400668160000001E-6</v>
@@ -5531,8 +5621,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>45510.431689814817</v>
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5">
         <v>4.3990867599999999E-7</v>
@@ -5569,8 +5659,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>45512.469583333332</v>
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6">
         <v>1.0020410404E-5</v>
@@ -5610,8 +5700,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>45551.438842592594</v>
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
         <v>2.5388136147E-5</v>
@@ -5651,8 +5741,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>45559.396516203713</v>
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8">
         <v>8.3814024999999997E-8</v>
@@ -5692,8 +5782,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>45567.486678240741</v>
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9">
         <v>2.3793510563333328E-6</v>
@@ -5733,8 +5823,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>45575.428530092591</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10">
         <v>4.5658003333333333E-9</v>
@@ -5774,8 +5864,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>45577.514988425923</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11">
         <v>9.7380083333333341E-9</v>
@@ -5815,8 +5905,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>45581.431863425933</v>
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12">
         <v>3.0286341333333342E-8</v>
@@ -5856,8 +5946,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>45590.521087962959</v>
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13">
         <v>5.8637712133333332E-7</v>
@@ -5897,8 +5987,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>45636.426770833343</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14">
         <v>2.5805707230000001E-6</v>
@@ -5938,8 +6028,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>45695.437777777777</v>
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15">
         <v>5.1461829904000001E-5</v>
@@ -5976,8 +6066,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>45699.435034722221</v>
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16">
         <v>3.6442259105333327E-5</v>
@@ -6017,8 +6107,8 @@
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>45702.570150462961</v>
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17">
         <v>1.6750430741333339E-5</v>
@@ -6058,8 +6148,8 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>45709.443043981482</v>
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18">
         <v>8.1642003333333337E-7</v>
@@ -6099,8 +6189,8 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>45712.429942129631</v>
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19">
         <v>2.4703057633333328E-7</v>
@@ -6140,8 +6230,8 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>45749.684745370367</v>
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20">
         <v>6.1283064270000017E-6</v>
@@ -6181,8 +6271,8 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>45750.456342592603</v>
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21">
         <v>8.4170389453333348E-6</v>
@@ -6222,8 +6312,8 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>45751.463090277779</v>
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22">
         <v>3.6236887456333338E-5</v>
@@ -6263,8 +6353,8 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>45775.660162037027</v>
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23">
         <v>4.698691208999999E-5</v>
@@ -6304,8 +6394,8 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>45777.673206018517</v>
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24">
         <v>2.61242569E-6</v>
@@ -6345,8 +6435,8 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>45784.682685185187</v>
+      <c r="A25" t="s">
+        <v>36</v>
       </c>
       <c r="B25">
         <v>1.87005625E-6</v>
@@ -6386,8 +6476,8 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>45785.61341435185</v>
+      <c r="A26" t="s">
+        <v>37</v>
       </c>
       <c r="B26">
         <v>6.7272803999999989E-7</v>
@@ -6427,8 +6517,8 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>45786.607685185183</v>
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27">
         <v>5.3097984900000006E-6</v>
@@ -6468,8 +6558,8 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>45789.486319444448</v>
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28">
         <v>6.5484810000000006E-8</v>
@@ -6509,8 +6599,8 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>45790.532141203701</v>
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29">
         <v>2.0331081000000001E-7</v>
@@ -6550,8 +6640,8 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>45795.64603009259</v>
+      <c r="A30" t="s">
+        <v>41</v>
       </c>
       <c r="B30">
         <v>1.8404100000000001E-9</v>
@@ -6642,8 +6732,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>45497.456319444442</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0.33993099999999998</v>
@@ -6683,8 +6773,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>45502.568819444437</v>
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3">
         <v>0.18506900000000001</v>
@@ -6724,8 +6814,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>45506.432141203702</v>
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4">
         <v>0.27326400000000001</v>
@@ -6765,8 +6855,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>45510.431689814817</v>
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5">
         <v>0.30208299999999999</v>
@@ -6803,8 +6893,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>45512.469583333332</v>
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6">
         <v>0.35486099999999998</v>
@@ -6844,8 +6934,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>45551.438842592594</v>
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
         <v>0.61493100000000001</v>
@@ -6885,8 +6975,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>45559.396516203713</v>
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8">
         <v>0.16666700000000001</v>
@@ -6926,8 +7016,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>45567.486678240741</v>
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9">
         <v>0.46041700000000002</v>
@@ -6967,8 +7057,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>45575.428530092591</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10">
         <v>0.33541700000000002</v>
@@ -7008,8 +7098,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>45577.514988425923</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11">
         <v>0.39756900000000001</v>
@@ -7049,8 +7139,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>45581.431863425933</v>
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12">
         <v>0.51597199999999999</v>
@@ -7090,8 +7180,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>45590.521087962959</v>
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13">
         <v>0.48888900000000002</v>
@@ -7131,8 +7221,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>45636.426770833343</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14">
         <v>1.3819440000000001</v>
@@ -7172,8 +7262,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>45695.437777777777</v>
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15">
         <v>0.286111</v>
@@ -7210,8 +7300,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>45699.435034722221</v>
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16">
         <v>0.39687499999999998</v>
@@ -7251,8 +7341,8 @@
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>45702.570150462961</v>
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17">
         <v>0.27013900000000002</v>
@@ -7292,8 +7382,8 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>45709.443043981482</v>
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18">
         <v>0.137847</v>
@@ -7333,8 +7423,8 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>45712.429942129631</v>
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19">
         <v>0.26597199999999999</v>
@@ -7374,8 +7464,8 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>45749.684745370367</v>
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20">
         <v>6.9399999999999996E-4</v>
@@ -7415,8 +7505,8 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>45750.456342592603</v>
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21">
         <v>0.19722200000000001</v>
@@ -7456,8 +7546,8 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>45751.463090277779</v>
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22">
         <v>0.31979200000000002</v>
@@ -7497,8 +7587,8 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>45775.660162037027</v>
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23">
         <v>2.8819000000000001E-2</v>
@@ -7538,8 +7628,8 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>45777.673206018517</v>
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24">
         <v>0.19062499999999999</v>
@@ -7579,8 +7669,8 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>45784.682685185187</v>
+      <c r="A25" t="s">
+        <v>36</v>
       </c>
       <c r="B25">
         <v>0.16493099999999999</v>
@@ -7620,8 +7710,8 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>45785.61341435185</v>
+      <c r="A26" t="s">
+        <v>37</v>
       </c>
       <c r="B26">
         <v>1.042E-3</v>
@@ -7661,8 +7751,8 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>45786.607685185183</v>
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27">
         <v>0.202431</v>
@@ -7702,8 +7792,8 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>45789.486319444448</v>
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28">
         <v>5.2430999999999998E-2</v>
@@ -7743,8 +7833,8 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>45790.532141203701</v>
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29">
         <v>0.157639</v>
@@ -7784,8 +7874,8 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>45795.64603009259</v>
+      <c r="A30" t="s">
+        <v>41</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -7876,8 +7966,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>45497.456319444442</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
         <v>-1.2300000000000001E-4</v>
@@ -7917,8 +8007,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>45502.568819444437</v>
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3">
         <v>-3.19E-4</v>
@@ -7958,8 +8048,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>45506.432141203702</v>
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4">
         <v>-7.7000000000000001E-5</v>
@@ -7996,8 +8086,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>45510.431689814817</v>
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5">
         <v>-3.4999999999999997E-5</v>
@@ -8034,8 +8124,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>45512.469583333332</v>
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6">
         <v>-3.1300000000000002E-4</v>
@@ -8075,8 +8165,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>45551.438842592594</v>
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
         <v>-2.1800000000000001E-4</v>
@@ -8116,8 +8206,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>45559.396516203713</v>
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8">
         <v>-2.9E-5</v>
@@ -8154,8 +8244,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>45567.486678240741</v>
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9">
         <v>-2.22E-4</v>
@@ -8195,8 +8285,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>45575.428530092591</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10">
         <v>-2.0999999999999999E-5</v>
@@ -8236,8 +8326,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>45577.514988425923</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11">
         <v>-2.8E-5</v>
@@ -8277,8 +8367,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>45581.431863425933</v>
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12">
         <v>-4.0000000000000003E-5</v>
@@ -8318,8 +8408,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>45590.521087962959</v>
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13">
         <v>-1.11E-4</v>
@@ -8359,8 +8449,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>45636.426770833343</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14">
         <v>-1.8200000000000001E-4</v>
@@ -8400,8 +8490,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>45695.437777777777</v>
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15">
         <v>-2.4899999999999998E-4</v>
@@ -8438,8 +8528,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>45699.435034722221</v>
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16">
         <v>-1.2899999999999999E-4</v>
@@ -8479,8 +8569,8 @@
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>45702.570150462961</v>
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17">
         <v>-3.3399999999999999E-4</v>
@@ -8520,8 +8610,8 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>45709.443043981482</v>
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18">
         <v>-1.54E-4</v>
@@ -8561,8 +8651,8 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>45712.429942129631</v>
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19">
         <v>-6.0999999999999999E-5</v>
@@ -8602,8 +8692,8 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>45749.684745370367</v>
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20">
         <v>-1.8309999999999999E-3</v>
@@ -8643,8 +8733,8 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>45750.456342592603</v>
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21">
         <v>-3.4200000000000002E-4</v>
@@ -8684,8 +8774,8 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>45751.463090277779</v>
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22">
         <v>-1.95E-4</v>
@@ -8725,8 +8815,8 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>45775.660162037027</v>
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23">
         <v>-1.4069999999999999E-2</v>
@@ -8766,8 +8856,8 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>45777.673206018517</v>
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24">
         <v>-6.2000000000000003E-5</v>
@@ -8807,8 +8897,8 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>45784.682685185187</v>
+      <c r="A25" t="s">
+        <v>36</v>
       </c>
       <c r="B25">
         <v>-3.0000000000000001E-5</v>
@@ -8848,8 +8938,8 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>45785.61341435185</v>
+      <c r="A26" t="s">
+        <v>37</v>
       </c>
       <c r="B26">
         <v>-1.63E-4</v>
@@ -8889,8 +8979,8 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>45786.607685185183</v>
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27">
         <v>-4.3000000000000002E-5</v>
@@ -8930,8 +9020,8 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>45789.486319444448</v>
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28">
         <v>-1.5E-5</v>
@@ -8968,8 +9058,8 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>45790.532141203701</v>
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29">
         <v>-2.0999999999999999E-5</v>
@@ -9009,8 +9099,8 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>45795.64603009259</v>
+      <c r="A30" t="s">
+        <v>41</v>
       </c>
       <c r="B30">
         <v>-3.9999999999999998E-6</v>
@@ -9058,10 +9148,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.6640625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -9105,8 +9191,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>45497.456319444442</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
         <v>3.891</v>
@@ -9146,8 +9232,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>45502.568819444437</v>
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3">
         <v>0.58499999999999996</v>
@@ -9187,8 +9273,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>45506.432141203702</v>
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4">
         <v>0.26100000000000001</v>
@@ -9228,8 +9314,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>45510.431689814817</v>
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5">
         <v>4.9000000000000002E-2</v>
@@ -9269,8 +9355,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>45512.469583333332</v>
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6">
         <v>1.046</v>
@@ -9310,8 +9396,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>45551.438842592594</v>
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
         <v>2.665</v>
@@ -9351,8 +9437,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>45559.396516203713</v>
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8">
         <v>1.2E-2</v>
@@ -9392,8 +9478,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>45567.486678240741</v>
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9">
         <v>0.161</v>
@@ -9433,8 +9519,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>45575.428530092591</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10">
         <v>4.0000000000000001E-3</v>
@@ -9474,8 +9560,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>45577.514988425923</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11">
         <v>2.1000000000000001E-2</v>
@@ -9515,8 +9601,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>45581.431863425933</v>
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12">
         <v>5.1999999999999998E-2</v>
@@ -9556,8 +9642,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>45590.521087962959</v>
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13">
         <v>0.27400000000000002</v>
@@ -9597,8 +9683,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>45636.426770833343</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14">
         <v>0.34899999999999998</v>
@@ -9638,8 +9724,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>45695.437777777777</v>
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15">
         <v>7.524</v>
@@ -9679,8 +9765,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>45699.435034722221</v>
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16">
         <v>5.2910000000000004</v>
@@ -9720,8 +9806,8 @@
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>45702.570150462961</v>
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17">
         <v>1.58</v>
@@ -9761,8 +9847,8 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>45709.443043981482</v>
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18">
         <v>8.8999999999999996E-2</v>
@@ -9802,8 +9888,8 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>45712.429942129631</v>
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19">
         <v>4.3999999999999997E-2</v>
@@ -9843,8 +9929,8 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>45749.684745370367</v>
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20">
         <v>0.26900000000000002</v>
@@ -9884,8 +9970,8 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>45750.456342592603</v>
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21">
         <v>0.48099999999999998</v>
@@ -9925,8 +10011,8 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>45751.463090277779</v>
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22">
         <v>4.2439999999999998</v>
@@ -9966,8 +10052,8 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>45775.660162037027</v>
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23">
         <v>0.58799999999999997</v>
@@ -10007,8 +10093,8 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>45777.673206018517</v>
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24">
         <v>0.13800000000000001</v>
@@ -10048,8 +10134,8 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>45784.682685185187</v>
+      <c r="A25" t="s">
+        <v>36</v>
       </c>
       <c r="B25">
         <v>9.9000000000000005E-2</v>
@@ -10089,8 +10175,8 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>45785.61341435185</v>
+      <c r="A26" t="s">
+        <v>37</v>
       </c>
       <c r="B26">
         <v>0.03</v>
@@ -10130,8 +10216,8 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>45786.607685185183</v>
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27">
         <v>0.39200000000000002</v>
@@ -10171,8 +10257,8 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>45789.486319444448</v>
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28">
         <v>3.0000000000000001E-3</v>
@@ -10212,8 +10298,8 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>45790.532141203701</v>
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29">
         <v>8.0000000000000002E-3</v>
@@ -10253,8 +10339,8 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>45795.64603009259</v>
+      <c r="A30" t="s">
+        <v>41</v>
       </c>
       <c r="B30">
         <v>0</v>

</xml_diff>

<commit_message>
time series data for COD events and associated timestamps stored in fetaure data set
</commit_message>
<xml_diff>
--- a/mfc_features.xlsx
+++ b/mfc_features.xlsx
@@ -7292,7 +7292,9 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
@@ -7720,7 +7722,9 @@
       <c r="H15" t="n">
         <v>150.226</v>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
       <c r="J15" t="n">
         <v>210.285</v>
       </c>
@@ -8616,7 +8620,9 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
@@ -9044,7 +9050,9 @@
       <c r="H15" t="n">
         <v>2.2567851076e-05</v>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
       <c r="J15" t="n">
         <v>4.4219781225e-05</v>
       </c>
@@ -9940,7 +9948,9 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
@@ -10368,7 +10378,9 @@
       <c r="H15" t="n">
         <v>128.108</v>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
       <c r="J15" t="n">
         <v>210.285</v>
       </c>
@@ -11264,7 +11276,9 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
@@ -11692,7 +11706,9 @@
       <c r="H15" t="n">
         <v>1.6411659664e-05</v>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
       <c r="J15" t="n">
         <v>4.4219781225e-05</v>
       </c>
@@ -12586,20 +12602,22 @@
         <v>0.000347</v>
       </c>
       <c r="H5" t="n">
-        <v>0.000347</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
       <c r="J5" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -12698,10 +12716,10 @@
         <v>0.166667</v>
       </c>
       <c r="C8" t="n">
-        <v>0.003472</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.003472</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0.111111</v>
@@ -12713,22 +12731,22 @@
         <v>0.246528</v>
       </c>
       <c r="H8" t="n">
-        <v>0.003472</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
         <v>0.100694</v>
       </c>
       <c r="J8" t="n">
-        <v>0.003472</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
         <v>0.003472</v>
       </c>
       <c r="L8" t="n">
-        <v>0.003472</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.003472</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -12784,10 +12802,10 @@
         <v>0.249653</v>
       </c>
       <c r="C10" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
         <v>0.249653</v>
@@ -12814,7 +12832,7 @@
         <v>0.13125</v>
       </c>
       <c r="M10" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -12867,13 +12885,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0.133681</v>
@@ -12882,25 +12900,25 @@
         <v>0.249653</v>
       </c>
       <c r="G12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -12943,7 +12961,7 @@
         <v>0.249653</v>
       </c>
       <c r="M13" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -12953,22 +12971,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
         <v>0.249653</v>
@@ -12980,13 +12998,13 @@
         <v>0.249653</v>
       </c>
       <c r="K14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -13016,7 +13034,9 @@
       <c r="H15" t="n">
         <v>0.046528</v>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
       <c r="J15" t="n">
         <v>0.249653</v>
       </c>
@@ -13285,7 +13305,7 @@
         <v>0.126736</v>
       </c>
       <c r="M21" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -13500,7 +13520,7 @@
         <v>0.089931</v>
       </c>
       <c r="M26" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -13559,7 +13579,7 @@
         <v>0.000347</v>
       </c>
       <c r="D28" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
         <v>0.001389</v>
@@ -13571,22 +13591,22 @@
         <v>0.249653</v>
       </c>
       <c r="H28" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
         <v>0.040625</v>
       </c>
       <c r="J28" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>0.000347</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">

</xml_diff>